<commit_message>
fix(genomics): ingest xlsx riconosce header '# rsid' e normalizza chrom/pos float (formato reale 23andMe)
La funzione _rows_xlsx ora:
- normalizza l'intestazione rimuovendo "#" prima di rsid
- converte chromosome/position da float a stringhe/int (1.0 → "1", 2000.0 → 2000)
- usa il nuovo helper _clean_num per normalizzazione consistente

Fixture aggiornato con header reale "# rsid" e dati numerici come float per rispecchiare il formato 23andMe autentico.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/genomics/scripts/tests/fixtures/sample.xlsx
+++ b/genomics/scripts/tests/fixtures/sample.xlsx
@@ -426,7 +426,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rsid</t>
+          <t># rsid</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -451,10 +451,8 @@
           <t>rs1000001</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B4" t="n">
+        <v>1</v>
       </c>
       <c r="C4" t="n">
         <v>1000</v>
@@ -471,10 +469,8 @@
           <t>rs1000002</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B5" t="n">
+        <v>1</v>
       </c>
       <c r="C5" t="n">
         <v>2000</v>
@@ -491,10 +487,8 @@
           <t>rs1000009</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B6" t="n">
+        <v>3</v>
       </c>
       <c r="C6" t="n">
         <v>9000</v>

</xml_diff>